<commit_message>
Zaid Alam - Full Stack Developer
</commit_message>
<xml_diff>
--- a/uploads/email_list.xlsx
+++ b/uploads/email_list.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\sendmail-to-hr\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A9E2FEC-528A-4C62-B4EE-303944B16B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93783425-4E22-4BD3-AEFC-1F35BDFD1CF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{7E36696A-FE27-4DB1-963D-1E74602D89D7}"/>
   </bookViews>
@@ -30,10 +30,10 @@
     <t>email</t>
   </si>
   <si>
-    <t>zaidalam010@gmail.com</t>
+    <t>zaidxxxxxx@gmail.com</t>
   </si>
   <si>
-    <t>bsk.badshahkhan@gmail.com</t>
+    <t>xxxxxxxxx@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -416,8 +416,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{7CB14D3A-AE0A-4809-9AD4-803794CFC462}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{5B69D3AE-4D78-4DAE-B6ED-05010E883EBC}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{5B69D3AE-4D78-4DAE-B6ED-05010E883EBC}"/>
+    <hyperlink ref="A2" r:id="rId2" xr:uid="{7CB14D3A-AE0A-4809-9AD4-803794CFC462}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>